<commit_message>
Ground demo assistant in actual reconciliation cases and record complete acceptance expectations
</commit_message>
<xml_diff>
--- a/demo bills/naturelabs1/EXPECTED_RESULTS.xlsx
+++ b/demo bills/naturelabs1/EXPECTED_RESULTS.xlsx
@@ -10,7 +10,9 @@
     <sheet name="Invoices" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Expected KPIs" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Signed totals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Expected reports" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Reconciliation" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Assumptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1931,6 +1933,222 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:B12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Report</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Expected rows</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>liability</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>without_itc</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>pending</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>mismatches</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>unmatched</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>purchases</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Without ITC: non-eligible purchase value</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>11038.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Without ITC: eligible classification but credit not established</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>36763.12</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Classification</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Exact</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Amount/head mismatch</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Unsupported purchase credit note</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Books only</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Statement only</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>